<commit_message>
Correct electricity-factor and RER wording from second review
- Caveat 2.4: list the electricity factor by year, say that only main
  and secondary space heating and main water heating are stored at
  primary / 2.08 (supplementary water used the factor in force up to
  2012), and give the real primary/delivered ratios of other fuels.
- Caveat 2.3: note the 2008-12 certificates whose declared secondary
  heating has no fuel, so DEAP gave it delivered energy but no primary
  energy or CO2; print their count by year.
- Definitions: RER coverage by period; delivered energy note.

No exported figures change.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gu3i4cJvPDofubpZEf7gqJ
</commit_message>
<xml_diff>
--- a/outputs/ber_results_by_type_and_band.xlsx
+++ b/outputs/ber_results_by_type_and_band.xlsx
@@ -11693,7 +11693,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>DEAP-calculated delivered energy for space heating, water heating, lighting and pumps/fans under standard occupancy, before deducting on-site PV; appliances and cooking are not included. Electric heating end uses are rebuilt as primary energy / the electricity factor in force (the file stores primary / 2.08)</t>
+          <t>DEAP-calculated delivered energy for space heating, water heating, lighting and pumps/fans under standard occupancy, before deducting on-site PV; appliances and cooking are not included. Electric heating end uses are rebuilt as primary energy / the electricity factor in force (the file stores most electric heating as primary / 2.08)</t>
         </is>
       </c>
     </row>
@@ -11931,7 +11931,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Renewable Energy Ratio, filled from Nov 2019 only</t>
+          <t>Renewable Energy Ratio. Filled for all certificates assessed from 2021 and most assessed from Dec 2019, but missing for most assessed in Nov 2019 and Aug-Nov 2020; statistics use certificates that have it (base = rer_n)</t>
         </is>
       </c>
     </row>

</xml_diff>